<commit_message>
Update on caso práctico tema 3
</commit_message>
<xml_diff>
--- a/content/Ingeniería de Telecomunicación/Realización de proyectos de ICT/Servicios de radio y TV/Caso_Practico_Tema_3.xlsx
+++ b/content/Ingeniería de Telecomunicación/Realización de proyectos de ICT/Servicios de radio y TV/Caso_Practico_Tema_3.xlsx
@@ -8,9 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\palfa\Documents\GitHub\palfaros-knowledge-base\content\Ingeniería de Telecomunicación\Realización de proyectos de ICT\Servicios de radio y TV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55CE1041-2FDF-4573-A453-863F7FD080DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A5C54B0-9571-40C9-A8BC-81AAF147EFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" firstSheet="1" activeTab="2" xr2:uid="{05F20D0D-700A-40D6-B3B2-C08799F32B6C}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" firstSheet="1" activeTab="1" xr2:uid="{05F20D0D-700A-40D6-B3B2-C08799F32B6C}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" firstSheet="1" activeTab="2" xr2:uid="{25218655-3AA3-4A01-86F5-3FD4FD14765A}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="1" r:id="rId1"/>
@@ -429,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -441,9 +442,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2293,15 +2291,15 @@
     </row>
     <row r="100" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D100" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F100" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G100" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="101" spans="3:7" x14ac:dyDescent="0.25">
@@ -2370,11 +2368,11 @@
       </c>
       <c r="F105" s="3">
         <f>SUM(F97:F104)</f>
-        <v>37.306799999999996</v>
+        <v>41.306799999999996</v>
       </c>
       <c r="G105" s="3">
         <f>SUM(G97:G104)</f>
-        <v>37.933499999999995</v>
+        <v>41.933500000000002</v>
       </c>
     </row>
     <row r="106" spans="3:7" x14ac:dyDescent="0.25">
@@ -2431,15 +2429,15 @@
     </row>
     <row r="110" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D110" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F110" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G110" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="111" spans="3:7" x14ac:dyDescent="0.25">
@@ -2508,11 +2506,11 @@
       </c>
       <c r="F115" s="3">
         <f>SUM(F107:F114)</f>
-        <v>36.372</v>
+        <v>40.371999999999993</v>
       </c>
       <c r="G115" s="3">
         <f>SUM(G107:G114)</f>
-        <v>36.765000000000001</v>
+        <v>40.765000000000001</v>
       </c>
     </row>
     <row r="116" spans="3:7" x14ac:dyDescent="0.25">
@@ -2569,15 +2567,15 @@
     </row>
     <row r="120" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D120" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F120" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G120" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="121" spans="3:7" x14ac:dyDescent="0.25">
@@ -2646,11 +2644,11 @@
       </c>
       <c r="F125" s="3">
         <f>SUM(F117:F124)</f>
-        <v>36.596399999999996</v>
+        <v>40.596399999999996</v>
       </c>
       <c r="G125" s="3">
         <f>SUM(G117:G124)</f>
-        <v>37.045499999999997</v>
+        <v>41.045500000000004</v>
       </c>
     </row>
     <row r="126" spans="3:7" x14ac:dyDescent="0.25">
@@ -2707,15 +2705,15 @@
     </row>
     <row r="130" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D130" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F130" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G130" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="131" spans="3:7" x14ac:dyDescent="0.25">
@@ -2784,11 +2782,11 @@
       </c>
       <c r="F135" s="3">
         <f>SUM(F127:F134)</f>
-        <v>36.565199999999997</v>
+        <v>40.565199999999997</v>
       </c>
       <c r="G135" s="3">
         <f>SUM(G127:G134)</f>
-        <v>37.006499999999996</v>
+        <v>41.006500000000003</v>
       </c>
     </row>
     <row r="136" spans="3:7" x14ac:dyDescent="0.25">
@@ -2845,15 +2843,15 @@
     </row>
     <row r="140" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D140" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F140" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G140" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="141" spans="3:7" x14ac:dyDescent="0.25">
@@ -2922,11 +2920,11 @@
       </c>
       <c r="F145" s="3">
         <f>SUM(F137:F144)</f>
-        <v>36.4176</v>
+        <v>40.417599999999993</v>
       </c>
       <c r="G145" s="3">
         <f>SUM(G137:G144)</f>
-        <v>36.821999999999996</v>
+        <v>40.822000000000003</v>
       </c>
     </row>
     <row r="146" spans="2:7" x14ac:dyDescent="0.25">
@@ -2988,15 +2986,15 @@
     </row>
     <row r="151" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D151" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F151" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G151" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="152" spans="2:7" x14ac:dyDescent="0.25">
@@ -3065,11 +3063,11 @@
       </c>
       <c r="F156" s="3">
         <f>SUM(F148:F155)</f>
-        <v>32.544799999999995</v>
+        <v>36.544799999999995</v>
       </c>
       <c r="G156" s="3">
         <f>SUM(G148:G155)</f>
-        <v>32.980999999999995</v>
+        <v>36.981000000000002</v>
       </c>
     </row>
     <row r="157" spans="2:7" x14ac:dyDescent="0.25">
@@ -3126,15 +3124,15 @@
     </row>
     <row r="161" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D161" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F161" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G161" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="162" spans="3:7" x14ac:dyDescent="0.25">
@@ -3203,11 +3201,11 @@
       </c>
       <c r="F166" s="3">
         <f>SUM(F158:F165)</f>
-        <v>32.628799999999998</v>
+        <v>36.628799999999998</v>
       </c>
       <c r="G166" s="3">
         <f>SUM(G158:G165)</f>
-        <v>33.085999999999999</v>
+        <v>37.085999999999999</v>
       </c>
     </row>
     <row r="167" spans="3:7" x14ac:dyDescent="0.25">
@@ -3264,15 +3262,15 @@
     </row>
     <row r="171" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D171" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F171" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G171" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="172" spans="3:7" x14ac:dyDescent="0.25">
@@ -3341,11 +3339,11 @@
       </c>
       <c r="F176" s="3">
         <f>SUM(F168:F175)</f>
-        <v>33.179599999999994</v>
+        <v>37.179600000000001</v>
       </c>
       <c r="G176" s="3">
         <f>SUM(G168:G175)</f>
-        <v>33.774500000000003</v>
+        <v>37.774499999999996</v>
       </c>
     </row>
     <row r="177" spans="2:7" x14ac:dyDescent="0.25">
@@ -3402,15 +3400,15 @@
     </row>
     <row r="181" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D181" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F181" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G181" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="182" spans="2:7" x14ac:dyDescent="0.25">
@@ -3479,11 +3477,11 @@
       </c>
       <c r="F186" s="3">
         <f>SUM(F178:F185)</f>
-        <v>33.204799999999999</v>
+        <v>37.204799999999999</v>
       </c>
       <c r="G186" s="3">
         <f>SUM(G178:G185)</f>
-        <v>33.805999999999997</v>
+        <v>37.805999999999997</v>
       </c>
     </row>
     <row r="187" spans="2:7" x14ac:dyDescent="0.25">
@@ -3545,15 +3543,15 @@
     </row>
     <row r="192" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D192" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F192" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G192" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="193" spans="3:7" x14ac:dyDescent="0.25">
@@ -3622,11 +3620,11 @@
       </c>
       <c r="F197" s="3">
         <f>SUM(F189:F196)</f>
-        <v>37.166399999999996</v>
+        <v>41.166399999999996</v>
       </c>
       <c r="G197" s="3">
         <f>SUM(G189:G196)</f>
-        <v>37.757999999999996</v>
+        <v>41.757999999999996</v>
       </c>
     </row>
     <row r="198" spans="3:7" x14ac:dyDescent="0.25">
@@ -3683,15 +3681,15 @@
     </row>
     <row r="202" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D202" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F202" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G202" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="203" spans="3:7" x14ac:dyDescent="0.25">
@@ -3760,11 +3758,11 @@
       </c>
       <c r="F207" s="3">
         <f>SUM(F199:F206)</f>
-        <v>36.6</v>
+        <v>40.6</v>
       </c>
       <c r="G207" s="3">
         <f>SUM(G199:G206)</f>
-        <v>37.049999999999997</v>
+        <v>41.05</v>
       </c>
     </row>
     <row r="208" spans="3:7" x14ac:dyDescent="0.25">
@@ -3821,15 +3819,15 @@
     </row>
     <row r="212" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D212" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F212" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G212" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="213" spans="3:7" x14ac:dyDescent="0.25">
@@ -3898,11 +3896,11 @@
       </c>
       <c r="F217" s="3">
         <f>SUM(F209:F216)</f>
-        <v>36.964799999999997</v>
+        <v>40.964799999999997</v>
       </c>
       <c r="G217" s="3">
         <f>SUM(G209:G216)</f>
-        <v>37.505999999999993</v>
+        <v>41.505999999999993</v>
       </c>
     </row>
     <row r="218" spans="3:7" x14ac:dyDescent="0.25">
@@ -3959,15 +3957,15 @@
     </row>
     <row r="222" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D222" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F222" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G222" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="223" spans="3:7" x14ac:dyDescent="0.25">
@@ -4036,11 +4034,11 @@
       </c>
       <c r="F227" s="3">
         <f>SUM(F219:F226)</f>
-        <v>37.103999999999999</v>
+        <v>41.103999999999999</v>
       </c>
       <c r="G227" s="3">
         <f>SUM(G219:G226)</f>
-        <v>37.679999999999993</v>
+        <v>41.679999999999993</v>
       </c>
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.25">
@@ -4097,15 +4095,15 @@
     </row>
     <row r="232" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D232" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F232" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G232" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.25">
@@ -4174,11 +4172,11 @@
       </c>
       <c r="F237" s="3">
         <f>SUM(F229:F236)</f>
-        <v>37.297199999999997</v>
+        <v>41.297199999999997</v>
       </c>
       <c r="G237" s="3">
         <f>SUM(G229:G236)</f>
-        <v>37.921499999999995</v>
+        <v>41.921499999999995</v>
       </c>
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.25">
@@ -10645,15 +10643,15 @@
     </row>
     <row r="100" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D100" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F100" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G100" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="101" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -10722,11 +10720,11 @@
       </c>
       <c r="F105" s="3">
         <f>SUM(F97:F104)</f>
-        <v>37.306799999999996</v>
+        <v>41.306799999999996</v>
       </c>
       <c r="G105" s="3">
         <f>SUM(G97:G104)</f>
-        <v>37.933499999999995</v>
+        <v>41.933500000000002</v>
       </c>
     </row>
     <row r="106" spans="3:7" x14ac:dyDescent="0.25">
@@ -10783,15 +10781,15 @@
     </row>
     <row r="110" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D110" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F110" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G110" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="111" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -10860,11 +10858,11 @@
       </c>
       <c r="F115" s="3">
         <f>SUM(F107:F114)</f>
-        <v>36.372</v>
+        <v>40.371999999999993</v>
       </c>
       <c r="G115" s="3">
         <f>SUM(G107:G114)</f>
-        <v>36.765000000000001</v>
+        <v>40.765000000000001</v>
       </c>
     </row>
     <row r="116" spans="3:7" x14ac:dyDescent="0.25">
@@ -10921,15 +10919,15 @@
     </row>
     <row r="120" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D120" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F120" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G120" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="121" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -10998,11 +10996,11 @@
       </c>
       <c r="F125" s="3">
         <f>SUM(F117:F124)</f>
-        <v>36.596399999999996</v>
+        <v>40.596399999999996</v>
       </c>
       <c r="G125" s="3">
         <f>SUM(G117:G124)</f>
-        <v>37.045499999999997</v>
+        <v>41.045500000000004</v>
       </c>
     </row>
     <row r="126" spans="3:7" x14ac:dyDescent="0.25">
@@ -11059,15 +11057,15 @@
     </row>
     <row r="130" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D130" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F130" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G130" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="131" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -11136,11 +11134,11 @@
       </c>
       <c r="F135" s="3">
         <f>SUM(F127:F134)</f>
-        <v>36.565199999999997</v>
+        <v>40.565199999999997</v>
       </c>
       <c r="G135" s="3">
         <f>SUM(G127:G134)</f>
-        <v>37.006499999999996</v>
+        <v>41.006500000000003</v>
       </c>
     </row>
     <row r="136" spans="3:7" x14ac:dyDescent="0.25">
@@ -11197,15 +11195,15 @@
     </row>
     <row r="140" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D140" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F140" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G140" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="141" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -11274,11 +11272,11 @@
       </c>
       <c r="F145" s="3">
         <f>SUM(F137:F144)</f>
-        <v>36.4176</v>
+        <v>40.417599999999993</v>
       </c>
       <c r="G145" s="3">
         <f>SUM(G137:G144)</f>
-        <v>36.821999999999996</v>
+        <v>40.822000000000003</v>
       </c>
     </row>
     <row r="146" spans="2:7" x14ac:dyDescent="0.25">
@@ -11340,15 +11338,15 @@
     </row>
     <row r="151" spans="2:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D151" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F151" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G151" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="152" spans="2:7" hidden="1" x14ac:dyDescent="0.25">
@@ -11417,11 +11415,11 @@
       </c>
       <c r="F156" s="4">
         <f>SUM(F148:F155)</f>
-        <v>32.544799999999995</v>
-      </c>
-      <c r="G156" s="5">
+        <v>36.544799999999995</v>
+      </c>
+      <c r="G156" s="3">
         <f>SUM(G148:G155)</f>
-        <v>32.980999999999995</v>
+        <v>36.981000000000002</v>
       </c>
     </row>
     <row r="157" spans="2:7" x14ac:dyDescent="0.25">
@@ -11478,15 +11476,15 @@
     </row>
     <row r="161" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D161" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F161" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G161" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="162" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -11555,11 +11553,11 @@
       </c>
       <c r="F166" s="3">
         <f>SUM(F158:F165)</f>
-        <v>32.628799999999998</v>
+        <v>36.628799999999998</v>
       </c>
       <c r="G166" s="3">
         <f>SUM(G158:G165)</f>
-        <v>33.085999999999999</v>
+        <v>37.085999999999999</v>
       </c>
     </row>
     <row r="167" spans="3:7" x14ac:dyDescent="0.25">
@@ -11616,15 +11614,15 @@
     </row>
     <row r="171" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D171" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F171" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G171" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="172" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -11693,11 +11691,11 @@
       </c>
       <c r="F176" s="3">
         <f>SUM(F168:F175)</f>
-        <v>33.179599999999994</v>
+        <v>37.179600000000001</v>
       </c>
       <c r="G176" s="3">
         <f>SUM(G168:G175)</f>
-        <v>33.774500000000003</v>
+        <v>37.774499999999996</v>
       </c>
     </row>
     <row r="177" spans="2:7" x14ac:dyDescent="0.25">
@@ -11754,15 +11752,15 @@
     </row>
     <row r="181" spans="2:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D181" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F181" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G181" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="182" spans="2:7" hidden="1" x14ac:dyDescent="0.25">
@@ -11831,11 +11829,11 @@
       </c>
       <c r="F186" s="3">
         <f>SUM(F178:F185)</f>
-        <v>33.204799999999999</v>
+        <v>37.204799999999999</v>
       </c>
       <c r="G186" s="3">
         <f>SUM(G178:G185)</f>
-        <v>33.805999999999997</v>
+        <v>37.805999999999997</v>
       </c>
     </row>
     <row r="187" spans="2:7" x14ac:dyDescent="0.25">
@@ -11897,15 +11895,15 @@
     </row>
     <row r="192" spans="2:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D192" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F192" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G192" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="193" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -11974,11 +11972,11 @@
       </c>
       <c r="F197" s="3">
         <f>SUM(F189:F196)</f>
-        <v>37.166399999999996</v>
+        <v>41.166399999999996</v>
       </c>
       <c r="G197" s="3">
         <f>SUM(G189:G196)</f>
-        <v>37.757999999999996</v>
+        <v>41.757999999999996</v>
       </c>
     </row>
     <row r="198" spans="3:7" x14ac:dyDescent="0.25">
@@ -12035,15 +12033,15 @@
     </row>
     <row r="202" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D202" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F202" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G202" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="203" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -12112,11 +12110,11 @@
       </c>
       <c r="F207" s="3">
         <f>SUM(F199:F206)</f>
-        <v>36.6</v>
+        <v>40.6</v>
       </c>
       <c r="G207" s="3">
         <f>SUM(G199:G206)</f>
-        <v>37.049999999999997</v>
+        <v>41.05</v>
       </c>
     </row>
     <row r="208" spans="3:7" x14ac:dyDescent="0.25">
@@ -12173,15 +12171,15 @@
     </row>
     <row r="212" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D212" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F212" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G212" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="213" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -12250,11 +12248,11 @@
       </c>
       <c r="F217" s="3">
         <f>SUM(F209:F216)</f>
-        <v>36.964799999999997</v>
+        <v>40.964799999999997</v>
       </c>
       <c r="G217" s="3">
         <f>SUM(G209:G216)</f>
-        <v>37.505999999999993</v>
+        <v>41.505999999999993</v>
       </c>
     </row>
     <row r="218" spans="3:7" x14ac:dyDescent="0.25">
@@ -12311,15 +12309,15 @@
     </row>
     <row r="222" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D222" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F222" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G222" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="223" spans="3:7" hidden="1" x14ac:dyDescent="0.25">
@@ -12388,11 +12386,11 @@
       </c>
       <c r="F227" s="3">
         <f>SUM(F219:F226)</f>
-        <v>37.103999999999999</v>
+        <v>41.103999999999999</v>
       </c>
       <c r="G227" s="3">
         <f>SUM(G219:G226)</f>
-        <v>37.679999999999993</v>
+        <v>41.679999999999993</v>
       </c>
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.25">
@@ -12449,15 +12447,15 @@
     </row>
     <row r="232" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="D232" s="2" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F232" s="3">
-        <f>Datos!C$9</f>
-        <v>17</v>
+        <f>Datos!C$6</f>
+        <v>21</v>
       </c>
       <c r="G232" s="3">
-        <f>Datos!D$9</f>
-        <v>17</v>
+        <f>Datos!D$6</f>
+        <v>21</v>
       </c>
     </row>
     <row r="233" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
@@ -12526,11 +12524,11 @@
       </c>
       <c r="F237" s="3">
         <f>SUM(F229:F236)</f>
-        <v>37.297199999999997</v>
+        <v>41.297199999999997</v>
       </c>
       <c r="G237" s="3">
         <f>SUM(G229:G236)</f>
-        <v>37.921499999999995</v>
+        <v>41.921499999999995</v>
       </c>
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.25">
@@ -12702,7 +12700,7 @@
       <c r="D251" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F251" s="5">
+      <c r="F251" s="3">
         <f>SUM(F241:F250)</f>
         <v>40.948799999999999</v>
       </c>
@@ -16099,11 +16097,11 @@
       <c r="D496" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F496" s="5">
+      <c r="F496" s="3">
         <f>SUM(F484:F495)</f>
         <v>35.828800000000001</v>
       </c>
-      <c r="G496" s="5">
+      <c r="G496" s="3">
         <f>SUM(G484:G495)</f>
         <v>36.436</v>
       </c>

</xml_diff>